<commit_message>
data(nzd): monthly refresh 2026-09-15T09:15Z
</commit_message>
<xml_diff>
--- a/logs/nzd/raw/R1.xlsx
+++ b/logs/nzd/raw/R1.xlsx
@@ -14228,6 +14228,80 @@
         <v>73237</v>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" s="28">
+        <v>46265</v>
+      </c>
+      <c r="B187" s="16">
+        <v>14497</v>
+      </c>
+      <c r="C187" s="16">
+        <v>19249</v>
+      </c>
+      <c r="D187" s="16">
+        <v>6869</v>
+      </c>
+      <c r="E187" s="16">
+        <v>16057</v>
+      </c>
+      <c r="F187" s="16">
+        <v>11484</v>
+      </c>
+      <c r="G187" s="16">
+        <v>571</v>
+      </c>
+      <c r="H187" s="16">
+        <v>478</v>
+      </c>
+      <c r="I187" s="16">
+        <v>1317</v>
+      </c>
+      <c r="J187" s="16">
+        <v>145</v>
+      </c>
+      <c r="K187" s="16">
+        <v>70667</v>
+      </c>
+      <c r="L187" s="16">
+        <v>18441</v>
+      </c>
+      <c r="M187" s="16">
+        <v>53490</v>
+      </c>
+      <c r="N187" s="16">
+        <v>0</v>
+      </c>
+      <c r="O187" s="16">
+        <v>0</v>
+      </c>
+      <c r="P187" s="16">
+        <v>1309</v>
+      </c>
+      <c r="Q187" s="16">
+        <v>0</v>
+      </c>
+      <c r="R187" s="16">
+        <v>0</v>
+      </c>
+      <c r="S187" s="16">
+        <v>10200</v>
+      </c>
+      <c r="T187" s="16">
+        <v>129</v>
+      </c>
+      <c r="U187" s="16">
+        <v>21</v>
+      </c>
+      <c r="V187" s="16">
+        <v>65149</v>
+      </c>
+      <c r="W187" s="16">
+        <v>5518</v>
+      </c>
+      <c r="X187" s="16">
+        <v>70667</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B5" location="'Series Definitions'!R2C3"/>
@@ -14296,7 +14370,7 @@
         <v>57</v>
       </c>
       <c r="B4" s="27">
-        <v>46248</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="5"/>

</xml_diff>